<commit_message>
Complete Phase 2 read-only MCP integration and ISO Excel dates
</commit_message>
<xml_diff>
--- a/data/defensa_performance_demo.xlsx
+++ b/data/defensa_performance_demo.xlsx
@@ -14,61 +14,67 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="2">
-    <x:border/>
-    <x:border/>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="10">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="2">
+    <border/>
+    <border/>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0"/>
+  </cellStyles>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -348,7 +354,7 @@
       <x:c r="C2" s="7" t="str">
         <x:v>Lautaro Cabrera</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="n">
+      <x:c r="D2" s="10" t="n">
         <x:v>46040</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
@@ -399,7 +405,7 @@
       <x:c r="C3" s="7" t="str">
         <x:v>Mateo Acosta</x:v>
       </x:c>
-      <x:c r="D3" s="7" t="n">
+      <x:c r="D3" s="10" t="n">
         <x:v>46047</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
@@ -450,7 +456,7 @@
       <x:c r="C4" s="7" t="str">
         <x:v>Emiliano Correa</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="n">
+      <x:c r="D4" s="10" t="n">
         <x:v>46052</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
@@ -501,7 +507,7 @@
       <x:c r="C5" s="7" t="str">
         <x:v>Tomás Ferreyra</x:v>
       </x:c>
-      <x:c r="D5" s="7" t="n">
+      <x:c r="D5" s="10" t="n">
         <x:v>46061</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
@@ -552,7 +558,7 @@
       <x:c r="C6" s="7" t="str">
         <x:v>Ramiro Godoy</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="n">
+      <x:c r="D6" s="10" t="n">
         <x:v>46064</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
@@ -603,7 +609,7 @@
       <x:c r="C7" s="7" t="str">
         <x:v>Joaquín Sosa</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="n">
+      <x:c r="D7" s="10" t="n">
         <x:v>46069</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
@@ -654,7 +660,7 @@
       <x:c r="C8" s="7" t="str">
         <x:v>Franco Quiroga</x:v>
       </x:c>
-      <x:c r="D8" s="7" t="n">
+      <x:c r="D8" s="10" t="n">
         <x:v>46073</x:v>
       </x:c>
       <x:c r="E8" s="7" t="str">
@@ -705,7 +711,7 @@
       <x:c r="C9" s="7" t="str">
         <x:v>Santino López</x:v>
       </x:c>
-      <x:c r="D9" s="7" t="n">
+      <x:c r="D9" s="10" t="n">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="E9" s="7" t="str">
@@ -756,7 +762,7 @@
       <x:c r="C10" s="7" t="str">
         <x:v>Mateo Acosta</x:v>
       </x:c>
-      <x:c r="D10" s="7" t="n">
+      <x:c r="D10" s="10" t="n">
         <x:v>46086</x:v>
       </x:c>
       <x:c r="E10" s="7" t="str">
@@ -809,7 +815,7 @@
       <x:c r="C11" s="7" t="str">
         <x:v>Valentín Castro</x:v>
       </x:c>
-      <x:c r="D11" s="7" t="n">
+      <x:c r="D11" s="10" t="n">
         <x:v>46090</x:v>
       </x:c>
       <x:c r="E11" s="7" t="str">
@@ -860,7 +866,7 @@
       <x:c r="C12" s="7" t="str">
         <x:v>Federico Paz</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="n">
+      <x:c r="D12" s="10" t="n">
         <x:v>46095</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str">
@@ -911,7 +917,7 @@
       <x:c r="C13" s="7" t="str">
         <x:v>Tomás Ferreyra</x:v>
       </x:c>
-      <x:c r="D13" s="7" t="n">
+      <x:c r="D13" s="10" t="n">
         <x:v>46099</x:v>
       </x:c>
       <x:c r="E13" s="7" t="str">
@@ -964,7 +970,7 @@
       <x:c r="C14" s="7" t="str">
         <x:v>Ignacio Leiva</x:v>
       </x:c>
-      <x:c r="D14" s="7" t="n">
+      <x:c r="D14" s="10" t="n">
         <x:v>46103</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
@@ -1015,7 +1021,7 @@
       <x:c r="C15" s="7" t="str">
         <x:v>Bruno Medina</x:v>
       </x:c>
-      <x:c r="D15" s="7" t="n">
+      <x:c r="D15" s="10" t="n">
         <x:v>46114</x:v>
       </x:c>
       <x:c r="E15" s="7" t="str">
@@ -1066,7 +1072,7 @@
       <x:c r="C16" s="7" t="str">
         <x:v>Santino López</x:v>
       </x:c>
-      <x:c r="D16" s="7" t="n">
+      <x:c r="D16" s="10" t="n">
         <x:v>46123</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
@@ -1119,7 +1125,7 @@
       <x:c r="C17" s="7" t="str">
         <x:v>Thiago Roldán</x:v>
       </x:c>
-      <x:c r="D17" s="7" t="n">
+      <x:c r="D17" s="10" t="n">
         <x:v>46124</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
@@ -1170,7 +1176,7 @@
       <x:c r="C18" s="7" t="str">
         <x:v>Máximo Villalba</x:v>
       </x:c>
-      <x:c r="D18" s="7" t="n">
+      <x:c r="D18" s="10" t="n">
         <x:v>46132</x:v>
       </x:c>
       <x:c r="E18" s="7" t="str">
@@ -1221,7 +1227,7 @@
       <x:c r="C19" s="7" t="str">
         <x:v>Emiliano Correa</x:v>
       </x:c>
-      <x:c r="D19" s="7" t="n">
+      <x:c r="D19" s="10" t="n">
         <x:v>46137</x:v>
       </x:c>
       <x:c r="E19" s="7" t="str">
@@ -1274,7 +1280,7 @@
       <x:c r="C20" s="7" t="str">
         <x:v>Lautaro Cabrera</x:v>
       </x:c>
-      <x:c r="D20" s="7" t="n">
+      <x:c r="D20" s="10" t="n">
         <x:v>46139</x:v>
       </x:c>
       <x:c r="E20" s="7" t="str">
@@ -1327,7 +1333,7 @@
       <x:c r="C21" s="7" t="str">
         <x:v>Ramiro Godoy</x:v>
       </x:c>
-      <x:c r="D21" s="7" t="n">
+      <x:c r="D21" s="10" t="n">
         <x:v>46146</x:v>
       </x:c>
       <x:c r="E21" s="7" t="str">
@@ -1380,7 +1386,7 @@
       <x:c r="C22" s="7" t="str">
         <x:v>Lucas Benítez</x:v>
       </x:c>
-      <x:c r="D22" s="7" t="n">
+      <x:c r="D22" s="10" t="n">
         <x:v>46152</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str">
@@ -1431,7 +1437,7 @@
       <x:c r="C23" s="7" t="str">
         <x:v>Bautista Núñez</x:v>
       </x:c>
-      <x:c r="D23" s="7" t="n">
+      <x:c r="D23" s="10" t="n">
         <x:v>46159</x:v>
       </x:c>
       <x:c r="E23" s="7" t="str">
@@ -1482,7 +1488,7 @@
       <x:c r="C24" s="7" t="str">
         <x:v>Thiago Roldán</x:v>
       </x:c>
-      <x:c r="D24" s="7" t="n">
+      <x:c r="D24" s="10" t="n">
         <x:v>46164</x:v>
       </x:c>
       <x:c r="E24" s="7" t="str">
@@ -1535,7 +1541,7 @@
       <x:c r="C25" s="7" t="str">
         <x:v>Benjamín Toledo</x:v>
       </x:c>
-      <x:c r="D25" s="7" t="n">
+      <x:c r="D25" s="10" t="n">
         <x:v>46167</x:v>
       </x:c>
       <x:c r="E25" s="7" t="str">
@@ -1586,7 +1592,7 @@
       <x:c r="C26" s="7" t="str">
         <x:v>Nicolás Arce</x:v>
       </x:c>
-      <x:c r="D26" s="7" t="n">
+      <x:c r="D26" s="10" t="n">
         <x:v>46172</x:v>
       </x:c>
       <x:c r="E26" s="7" t="str">
@@ -1637,7 +1643,7 @@
       <x:c r="C27" s="7" t="str">
         <x:v>Agustín Vera</x:v>
       </x:c>
-      <x:c r="D27" s="7" t="n">
+      <x:c r="D27" s="10" t="n">
         <x:v>46176</x:v>
       </x:c>
       <x:c r="E27" s="7" t="str">
@@ -1688,7 +1694,7 @@
       <x:c r="C28" s="7" t="str">
         <x:v>Ignacio Leiva</x:v>
       </x:c>
-      <x:c r="D28" s="7" t="n">
+      <x:c r="D28" s="10" t="n">
         <x:v>46178</x:v>
       </x:c>
       <x:c r="E28" s="7" t="str">
@@ -1739,7 +1745,7 @@
       <x:c r="C29" s="7" t="str">
         <x:v>Lautaro Cabrera</x:v>
       </x:c>
-      <x:c r="D29" s="7" t="n">
+      <x:c r="D29" s="10" t="n">
         <x:v>46179</x:v>
       </x:c>
       <x:c r="E29" s="7" t="str">
@@ -1790,7 +1796,7 @@
       <x:c r="C30" s="7" t="str">
         <x:v>Mateo Acosta</x:v>
       </x:c>
-      <x:c r="D30" s="7" t="n">
+      <x:c r="D30" s="10" t="n">
         <x:v>46180</x:v>
       </x:c>
       <x:c r="E30" s="7" t="str">
@@ -1841,7 +1847,7 @@
       <x:c r="C31" s="7" t="str">
         <x:v>Franco Quiroga</x:v>
       </x:c>
-      <x:c r="D31" s="7" t="n">
+      <x:c r="D31" s="10" t="n">
         <x:v>46181</x:v>
       </x:c>
       <x:c r="E31" s="7" t="str">
@@ -1894,7 +1900,7 @@
       <x:c r="C32" s="7" t="str">
         <x:v>Federico Paz</x:v>
       </x:c>
-      <x:c r="D32" s="7" t="n">
+      <x:c r="D32" s="10" t="n">
         <x:v>46184</x:v>
       </x:c>
       <x:c r="E32" s="7" t="str">
@@ -1945,7 +1951,7 @@
       <x:c r="C33" s="7" t="str">
         <x:v>Valentín Castro</x:v>
       </x:c>
-      <x:c r="D33" s="7" t="n">
+      <x:c r="D33" s="10" t="n">
         <x:v>46185</x:v>
       </x:c>
       <x:c r="E33" s="7" t="str">
@@ -1996,7 +2002,7 @@
       <x:c r="C34" s="7" t="str">
         <x:v>Joaquín Sosa</x:v>
       </x:c>
-      <x:c r="D34" s="7" t="n">
+      <x:c r="D34" s="10" t="n">
         <x:v>46186</x:v>
       </x:c>
       <x:c r="E34" s="7" t="str">
@@ -2047,7 +2053,7 @@
       <x:c r="C35" s="7" t="str">
         <x:v>Gonzalo Mena</x:v>
       </x:c>
-      <x:c r="D35" s="7" t="n">
+      <x:c r="D35" s="10" t="n">
         <x:v>46188</x:v>
       </x:c>
       <x:c r="E35" s="7" t="str">
@@ -2098,7 +2104,7 @@
       <x:c r="C36" s="7" t="str">
         <x:v>Emiliano Correa</x:v>
       </x:c>
-      <x:c r="D36" s="7" t="n">
+      <x:c r="D36" s="10" t="n">
         <x:v>46190</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str">
@@ -2149,7 +2155,7 @@
       <x:c r="C37" s="7" t="str">
         <x:v>Facundo Peralta</x:v>
       </x:c>
-      <x:c r="D37" s="7" t="n">
+      <x:c r="D37" s="10" t="n">
         <x:v>46191</x:v>
       </x:c>
       <x:c r="E37" s="7" t="str">
@@ -2200,7 +2206,7 @@
       <x:c r="C38" s="7" t="str">
         <x:v>Ignacio Leiva</x:v>
       </x:c>
-      <x:c r="D38" s="7" t="n">
+      <x:c r="D38" s="10" t="n">
         <x:v>46192</x:v>
       </x:c>
       <x:c r="E38" s="7" t="str">
@@ -2253,7 +2259,7 @@
       <x:c r="C39" s="7" t="str">
         <x:v>Thiago Roldán</x:v>
       </x:c>
-      <x:c r="D39" s="7" t="n">
+      <x:c r="D39" s="10" t="n">
         <x:v>46192</x:v>
       </x:c>
       <x:c r="E39" s="7" t="str">
@@ -2304,7 +2310,7 @@
       <x:c r="C40" s="7" t="str">
         <x:v>Facundo Peralta</x:v>
       </x:c>
-      <x:c r="D40" s="7" t="n">
+      <x:c r="D40" s="10" t="n">
         <x:v>46194</x:v>
       </x:c>
       <x:c r="E40" s="7" t="str">
@@ -2355,7 +2361,7 @@
       <x:c r="C41" s="7" t="str">
         <x:v>Simón Lagos</x:v>
       </x:c>
-      <x:c r="D41" s="7" t="n">
+      <x:c r="D41" s="10" t="n">
         <x:v>46196</x:v>
       </x:c>
       <x:c r="E41" s="7" t="str">
@@ -2406,7 +2412,7 @@
       <x:c r="C42" s="7" t="str">
         <x:v>Máximo Villalba</x:v>
       </x:c>
-      <x:c r="D42" s="7" t="n">
+      <x:c r="D42" s="10" t="n">
         <x:v>46197</x:v>
       </x:c>
       <x:c r="E42" s="7" t="str">
@@ -2457,7 +2463,7 @@
       <x:c r="C43" s="7" t="str">
         <x:v>Bautista Núñez</x:v>
       </x:c>
-      <x:c r="D43" s="7" t="n">
+      <x:c r="D43" s="10" t="n">
         <x:v>46198</x:v>
       </x:c>
       <x:c r="E43" s="7" t="str">
@@ -2508,7 +2514,7 @@
       <x:c r="C44" s="7" t="str">
         <x:v>Alan Paredes</x:v>
       </x:c>
-      <x:c r="D44" s="7" t="n">
+      <x:c r="D44" s="10" t="n">
         <x:v>46204</x:v>
       </x:c>
       <x:c r="E44" s="7" t="str">
@@ -2559,7 +2565,7 @@
       <x:c r="C45" s="7" t="str">
         <x:v>Federico Paz</x:v>
       </x:c>
-      <x:c r="D45" s="7" t="n">
+      <x:c r="D45" s="10" t="n">
         <x:v>46205</x:v>
       </x:c>
       <x:c r="E45" s="7" t="str">
@@ -2612,7 +2618,7 @@
       <x:c r="C46" s="7" t="str">
         <x:v>Benjamín Toledo</x:v>
       </x:c>
-      <x:c r="D46" s="7" t="n">
+      <x:c r="D46" s="10" t="n">
         <x:v>46205</x:v>
       </x:c>
       <x:c r="E46" s="7" t="str">
@@ -2663,7 +2669,7 @@
       <x:c r="C47" s="7" t="str">
         <x:v>Agustín Vera</x:v>
       </x:c>
-      <x:c r="D47" s="7" t="n">
+      <x:c r="D47" s="10" t="n">
         <x:v>46206</x:v>
       </x:c>
       <x:c r="E47" s="7" t="str">
@@ -2714,7 +2720,7 @@
       <x:c r="C48" s="7" t="str">
         <x:v>Tomás Ferreyra</x:v>
       </x:c>
-      <x:c r="D48" s="7" t="n">
+      <x:c r="D48" s="10" t="n">
         <x:v>46207</x:v>
       </x:c>
       <x:c r="E48" s="7" t="str">
@@ -2765,7 +2771,7 @@
       <x:c r="C49" s="7" t="str">
         <x:v>Damián Funes</x:v>
       </x:c>
-      <x:c r="D49" s="7" t="n">
+      <x:c r="D49" s="10" t="n">
         <x:v>46211</x:v>
       </x:c>
       <x:c r="E49" s="7" t="str">
@@ -2816,7 +2822,7 @@
       <x:c r="C50" s="7" t="str">
         <x:v>Gonzalo Mena</x:v>
       </x:c>
-      <x:c r="D50" s="7" t="n">
+      <x:c r="D50" s="10" t="n">
         <x:v>46211</x:v>
       </x:c>
       <x:c r="E50" s="7" t="str">
@@ -2867,7 +2873,7 @@
       <x:c r="C51" s="7" t="str">
         <x:v>Santino López</x:v>
       </x:c>
-      <x:c r="D51" s="7" t="n">
+      <x:c r="D51" s="10" t="n">
         <x:v>46212</x:v>
       </x:c>
       <x:c r="E51" s="7" t="str">
@@ -2918,7 +2924,7 @@
       <x:c r="C52" s="7" t="str">
         <x:v>Lucas Benítez</x:v>
       </x:c>
-      <x:c r="D52" s="7" t="n">
+      <x:c r="D52" s="10" t="n">
         <x:v>46213</x:v>
       </x:c>
       <x:c r="E52" s="7" t="str">
@@ -2969,7 +2975,7 @@
       <x:c r="C53" s="7" t="str">
         <x:v>Jerónimo Suárez</x:v>
       </x:c>
-      <x:c r="D53" s="7" t="n">
+      <x:c r="D53" s="10" t="n">
         <x:v>46215</x:v>
       </x:c>
       <x:c r="E53" s="7" t="str">
@@ -3020,7 +3026,7 @@
       <x:c r="C54" s="7" t="str">
         <x:v>Jerónimo Suárez</x:v>
       </x:c>
-      <x:c r="D54" s="7" t="n">
+      <x:c r="D54" s="10" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="E54" s="7" t="str">
@@ -3071,7 +3077,7 @@
       <x:c r="C55" s="7" t="str">
         <x:v>Ramiro Godoy</x:v>
       </x:c>
-      <x:c r="D55" s="7" t="n">
+      <x:c r="D55" s="10" t="n">
         <x:v>46218</x:v>
       </x:c>
       <x:c r="E55" s="7" t="str">
@@ -3122,7 +3128,7 @@
       <x:c r="C56" s="7" t="str">
         <x:v>Bruno Medina</x:v>
       </x:c>
-      <x:c r="D56" s="7" t="n">
+      <x:c r="D56" s="10" t="n">
         <x:v>46219</x:v>
       </x:c>
       <x:c r="E56" s="7" t="str">
@@ -3173,7 +3179,7 @@
       <x:c r="C57" s="7" t="str">
         <x:v>Simón Lagos</x:v>
       </x:c>
-      <x:c r="D57" s="7" t="n">
+      <x:c r="D57" s="10" t="n">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="E57" s="7" t="str">
@@ -3224,7 +3230,7 @@
       <x:c r="C58" s="7" t="str">
         <x:v>Damián Funes</x:v>
       </x:c>
-      <x:c r="D58" s="7" t="n">
+      <x:c r="D58" s="10" t="n">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="E58" s="7" t="str">
@@ -3275,7 +3281,7 @@
       <x:c r="C59" s="7" t="str">
         <x:v>Nicolás Arce</x:v>
       </x:c>
-      <x:c r="D59" s="7" t="n">
+      <x:c r="D59" s="10" t="n">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="E59" s="7" t="str">
@@ -3326,7 +3332,7 @@
       <x:c r="C60" s="7" t="str">
         <x:v>Franco Quiroga</x:v>
       </x:c>
-      <x:c r="D60" s="7" t="n">
+      <x:c r="D60" s="10" t="n">
         <x:v>46225</x:v>
       </x:c>
       <x:c r="E60" s="7" t="str">

</xml_diff>

<commit_message>
Complete Performance AI context and visualization improvements
</commit_message>
<xml_diff>
--- a/data/defensa_performance_demo.xlsx
+++ b/data/defensa_performance_demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eventos" sheetId="1" r:id="Rd76f49da90e845ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jugadores" sheetId="2" r:id="R389dc297a0674661"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario" sheetId="3" r:id="R19805f95cdeb4a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eventos" sheetId="1" r:id="Rb8c69c7da0214bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jugadores" sheetId="2" r:id="Rff0b5a1d522b4fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario" sheetId="3" r:id="R6db8a84fb15b49cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,67 +14,71 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="2">
-    <font>
-      <sz val="11"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Carlito"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="2">
-    <border/>
-    <border/>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0"/>
-  </cellStyles>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
+  <x:fonts count="2">
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="2">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+  </x:fills>
+  <x:borders count="2">
+    <x:border/>
+    <x:border/>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="13">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -291,57 +295,57 @@
     <x:col min="17" max="17" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="64" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>ID_Evento</x:v>
+        <x:v>Identificador del evento registrado</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>ID_Jugador</x:v>
+        <x:v>Identificador del jugador</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Jugador</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Fecha</x:v>
+        <x:v>Fecha del evento registrado</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>Tipo_evento</x:v>
+        <x:v>Tipo de lesión o problema físico registrado</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>Zona</x:v>
+        <x:v>Zona del cuerpo afectada</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>Lado</x:v>
+        <x:v>Lado del cuerpo afectado</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>Diagnóstico</x:v>
+        <x:v>Diagnóstico de la lesión o problema físico</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>Gravedad</x:v>
+        <x:v>Gravedad de la lesión registrada</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
-        <x:v>Días_baja</x:v>
+        <x:v>Días sin disponibilidad plena tras el evento</x:v>
       </x:c>
       <x:c r="K1" s="6" t="str">
-        <x:v>Contexto</x:v>
+        <x:v>Actividad en la que ocurrió el evento</x:v>
       </x:c>
       <x:c r="L1" s="6" t="str">
-        <x:v>Días_desde_partido_previo</x:v>
+        <x:v>Días entre el partido anterior y el evento registrado</x:v>
       </x:c>
       <x:c r="M1" s="6" t="str">
-        <x:v>Minutos_últimos_28d</x:v>
+        <x:v>Minutos de partido jugados en los 28 días anteriores al evento</x:v>
       </x:c>
       <x:c r="N1" s="6" t="str">
-        <x:v>Partidos_últimos_28d</x:v>
+        <x:v>Partidos jugados en los 28 días anteriores al evento</x:v>
       </x:c>
       <x:c r="O1" s="6" t="str">
-        <x:v>Antecedente_misma_zona_12m</x:v>
+        <x:v>Lesión o problema previo en la misma zona en los últimos 12 meses</x:v>
       </x:c>
       <x:c r="P1" s="6" t="str">
-        <x:v>Días_desde_RTP_previo</x:v>
+        <x:v>Días desde el regreso a jugar tras la lesión anterior hasta este evento</x:v>
       </x:c>
       <x:c r="Q1" s="6" t="str">
-        <x:v>Observaciones</x:v>
+        <x:v>Observaciones sobre el evento registrado</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3389,21 +3393,21 @@
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="64" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>ID_Jugador</x:v>
+        <x:v>Identificador del jugador</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
         <x:v>Jugador</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>Edad</x:v>
+        <x:v>Edad del jugador (años)</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Posición</x:v>
+        <x:v>Posición del jugador en el campo</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>Pierna dominante</x:v>
+        <x:v>Pierna dominante del jugador</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3840,159 +3844,159 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="64" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>Campo</x:v>
+        <x:v>Nombre de la columna del Excel</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Descripción</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="7" t="str">
-        <x:v>ID_Evento</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
+        <x:v>Qué significa la columna</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="45" customHeight="1">
+      <x:c r="A2" s="12" t="str">
+        <x:v>Identificador del evento registrado</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
         <x:v>Identificador ficticio único del evento.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="7" t="str">
-        <x:v>ID_Jugador</x:v>
-      </x:c>
-      <x:c r="B3" s="7" t="str">
+    <x:row r="3" ht="45" customHeight="1">
+      <x:c r="A3" s="12" t="str">
+        <x:v>Identificador del jugador</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
         <x:v>Identificador ficticio único del jugador.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="7" t="str">
+    <x:row r="4" ht="45" customHeight="1">
+      <x:c r="A4" s="12" t="str">
         <x:v>Jugador</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B4" s="12" t="str">
         <x:v>Nombre completamente ficticio.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="7" t="str">
-        <x:v>Fecha</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="str">
-        <x:v>Fecha ficticia del evento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="7" t="str">
-        <x:v>Tipo_evento</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="str">
-        <x:v>Lesión, recaída, sobrecarga o traumatismo.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="7" t="str">
-        <x:v>Zona</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="str">
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Fecha del evento registrado</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Fecha ficticia en la que ocurrió el evento registrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Tipo de lesión o problema físico registrado</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>Clasificación del evento registrado: lesión, recaída (nueva lesión tras una anterior), sobrecarga o traumatismo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Zona del cuerpo afectada</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
         <x:v>Región corporal afectada.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="7" t="str">
-        <x:v>Lado</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="str">
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>Lado del cuerpo afectado</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
         <x:v>Lado corporal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="7" t="str">
-        <x:v>Diagnóstico</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="str">
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>Diagnóstico de la lesión o problema físico</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
         <x:v>Descripción médica simplificada y ficticia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="7" t="str">
-        <x:v>Gravedad</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="str">
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="12" t="str">
+        <x:v>Gravedad de la lesión registrada</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
         <x:v>Clasificación simplificada para la demo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="7" t="str">
-        <x:v>Días_baja</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="str">
-        <x:v>Días ficticios sin disponibilidad plena.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7" t="str">
-        <x:v>Contexto</x:v>
-      </x:c>
-      <x:c r="B12" s="7" t="str">
-        <x:v>Partido o entrenamiento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="7" t="str">
-        <x:v>Días_desde_partido_previo</x:v>
-      </x:c>
-      <x:c r="B13" s="7" t="str">
-        <x:v>Recuperación desde el partido anterior.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="7" t="str">
-        <x:v>Minutos_últimos_28d</x:v>
-      </x:c>
-      <x:c r="B14" s="7" t="str">
-        <x:v>Minutos oficiales acumulados por el jugador durante los 28 días anteriores al evento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="7" t="str">
-        <x:v>Partidos_últimos_28d</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>Cantidad de partidos en los que participó el jugador durante los 28 días anteriores al evento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="7" t="str">
-        <x:v>Antecedente_misma_zona_12m</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="str">
-        <x:v>Si existía un evento previo en la misma zona.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="7" t="str">
-        <x:v>Días_desde_RTP_previo</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="str">
-        <x:v>Días desde retorno al juego previo; vacío si no aplica.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7" t="str">
-        <x:v>Observaciones</x:v>
-      </x:c>
-      <x:c r="B18" s="7" t="str">
+    <x:row r="11" ht="45" customHeight="1">
+      <x:c r="A11" s="12" t="str">
+        <x:v>Días sin disponibilidad plena tras el evento</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>Cantidad de días en los que el jugador no tuvo disponibilidad plena después del evento registrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>Actividad en la que ocurrió el evento</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Indica si el evento registrado ocurrió en un partido o durante un entrenamiento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>Días entre el partido anterior y el evento registrado</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>Cantidad de días entre el partido anterior del jugador y la fecha del evento registrado (lesión, recaída u otro problema físico). No equivale necesariamente a días completos de descanso ni implica que el evento ocurrió en un partido.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>Minutos de partido jugados en los 28 días anteriores al evento</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Minutos oficiales de partido acumulados por el jugador durante los 28 días anteriores al evento registrado. No equivale necesariamente a minutos desde su regreso tras una lesión.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Partidos jugados en los 28 días anteriores al evento</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>Cantidad de partidos en los que participó el jugador durante los 28 días anteriores al evento registrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>Lesión o problema previo en la misma zona en los últimos 12 meses</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>Indica si existía un evento anterior en la misma zona corporal durante los 12 meses previos al evento registrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="45" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Días desde el regreso a jugar tras la lesión anterior hasta este evento</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>Cantidad de días transcurridos desde el regreso del jugador a la actividad de juego tras una lesión anterior hasta la fecha del evento registrado. No representa minutos jugados; vacío si no aplica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Observaciones sobre el evento registrado</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
         <x:v>Contexto breve del registro.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7" t="str">
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" s="12" t="str">
         <x:v>AVISO</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="str">
+      <x:c r="B19" s="12" t="str">
         <x:v>Dataset 100% ficticio para demo. No implica causalidad ni debe usarse para decisiones médicas.</x:v>
       </x:c>
     </x:row>

</xml_diff>